<commit_message>
Update xslope_design.xlsx sample input
Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/lem/files/xslope_design.xlsx
+++ b/docs/lem/files/xslope_design.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10613"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/lem/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3507667D-50EA-9A4E-8822-5A07A27F6F05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9AA747A-7DE0-5B4D-A106-354C45B36FD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14260" yWindow="1640" windowWidth="34200" windowHeight="20240" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
+    <workbookView xWindow="27700" yWindow="1900" windowWidth="34200" windowHeight="20240" activeTab="2" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="156" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="279" uniqueCount="154">
   <si>
     <t>X</t>
   </si>
@@ -390,9 +390,6 @@
     <t>d</t>
   </si>
   <si>
-    <t>ψ</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="12"/>
@@ -411,9 +408,6 @@
       </rPr>
       <t>(d)</t>
     </r>
-  </si>
-  <si>
-    <t>s(ψ)</t>
   </si>
   <si>
     <t>Piezometric Line 2</t>
@@ -661,7 +655,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -779,6 +773,11 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow (Body)"/>
     </font>
   </fonts>
   <fills count="16">
@@ -1075,19 +1074,19 @@
     <xf numFmtId="0" fontId="16" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -7943,7 +7942,7 @@
   <sheetData>
     <row r="1" spans="1:7" ht="32" x14ac:dyDescent="0.4">
       <c r="A1" s="7" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="3" spans="1:7" ht="19" x14ac:dyDescent="0.25">
@@ -7960,11 +7959,11 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="B7" s="43" t="s">
+      <c r="B7" s="44" t="s">
         <v>47</v>
       </c>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
+      <c r="C7" s="44"/>
+      <c r="D7" s="44"/>
       <c r="F7" s="15" t="s">
         <v>15</v>
       </c>
@@ -7980,10 +7979,10 @@
         <v>62.4</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="G8" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
@@ -8055,10 +8054,10 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="F15" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G15" t="s">
         <v>123</v>
-      </c>
-      <c r="G15" t="s">
-        <v>125</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
@@ -8072,18 +8071,18 @@
     <row r="17" spans="2:7" x14ac:dyDescent="0.2">
       <c r="B17" s="1"/>
       <c r="F17" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="18" spans="2:7" x14ac:dyDescent="0.2">
       <c r="F18" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="G18" s="9" t="s">
         <v>124</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="20" spans="2:7" x14ac:dyDescent="0.2">
@@ -8117,34 +8116,34 @@
         <v>25</v>
       </c>
       <c r="B2" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>104</v>
+      </c>
+      <c r="D2" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="C2" s="12" t="s">
+      <c r="E2" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="D2" s="12" t="s">
+      <c r="F2" s="32" t="s">
+        <v>108</v>
+      </c>
+      <c r="G2" s="33" t="s">
+        <v>113</v>
+      </c>
+      <c r="H2" s="32" t="s">
+        <v>111</v>
+      </c>
+      <c r="I2" s="32" t="s">
+        <v>112</v>
+      </c>
+      <c r="J2" s="33" t="s">
+        <v>101</v>
+      </c>
+      <c r="K2" s="33" t="s">
         <v>107</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="F2" s="32" t="s">
-        <v>110</v>
-      </c>
-      <c r="G2" s="33" t="s">
-        <v>115</v>
-      </c>
-      <c r="H2" s="32" t="s">
-        <v>113</v>
-      </c>
-      <c r="I2" s="32" t="s">
-        <v>114</v>
-      </c>
-      <c r="J2" s="33" t="s">
-        <v>103</v>
-      </c>
-      <c r="K2" s="33" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.2">
@@ -8403,7 +8402,7 @@
       <c r="K19" s="3"/>
       <c r="M19" s="31"/>
       <c r="N19" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.2">
@@ -8422,7 +8421,7 @@
       <c r="K20" s="3"/>
       <c r="M20" s="34"/>
       <c r="N20" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.2">
@@ -8484,27 +8483,27 @@
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B2" s="52" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="C2" s="52"/>
       <c r="E2" s="48" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F2" s="48"/>
       <c r="H2" s="48" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="I2" s="48"/>
       <c r="K2" s="48" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="L2" s="48"/>
       <c r="N2" s="48" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="O2" s="48"/>
       <c r="Q2" s="48" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="R2" s="48"/>
     </row>
@@ -8512,23 +8511,23 @@
       <c r="B3" s="52"/>
       <c r="C3" s="52"/>
       <c r="E3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F3" s="38"/>
       <c r="H3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I3" s="38"/>
       <c r="K3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L3" s="38"/>
       <c r="N3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="O3" s="38"/>
       <c r="Q3" s="37" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="R3" s="38"/>
     </row>
@@ -8878,27 +8877,27 @@
   <sheetData>
     <row r="2" spans="2:18" x14ac:dyDescent="0.2">
       <c r="B2" s="53" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C2" s="53"/>
       <c r="E2" s="49" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F2" s="49"/>
       <c r="H2" s="49" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="I2" s="49"/>
       <c r="K2" s="49" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="L2" s="49"/>
       <c r="N2" s="49" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="O2" s="49"/>
       <c r="Q2" s="49" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="R2" s="49"/>
     </row>
@@ -8906,23 +8905,23 @@
       <c r="B3" s="53"/>
       <c r="C3" s="53"/>
       <c r="E3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="F3" s="40"/>
       <c r="H3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="I3" s="40"/>
       <c r="K3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="L3" s="40"/>
       <c r="N3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="O3" s="40"/>
       <c r="Q3" s="39" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="R3" s="40"/>
     </row>
@@ -9288,7 +9287,7 @@
       <c r="E2"/>
       <c r="F2"/>
       <c r="J2" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="O2" s="6"/>
     </row>
@@ -9302,7 +9301,7 @@
       <c r="E3"/>
       <c r="F3"/>
       <c r="J3" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="K3" t="s">
         <v>59</v>
@@ -9328,10 +9327,10 @@
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="J5" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="K5" s="9" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="O5" s="14"/>
     </row>
@@ -9342,36 +9341,36 @@
       <c r="Q6" s="1"/>
     </row>
     <row r="7" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="C7" s="44" t="s">
+      <c r="C7" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="D7" s="44"/>
-      <c r="E7" s="44"/>
-      <c r="F7" s="44"/>
-      <c r="G7" s="44"/>
-      <c r="H7" s="44"/>
-      <c r="I7" s="44"/>
-      <c r="J7" s="44"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
+      <c r="F7" s="43"/>
+      <c r="G7" s="43"/>
+      <c r="H7" s="43"/>
+      <c r="I7" s="43"/>
+      <c r="J7" s="43"/>
       <c r="K7" s="1"/>
-      <c r="L7" s="44" t="s">
+      <c r="L7" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="M7" s="44"/>
-      <c r="N7" s="44"/>
-      <c r="O7" s="44"/>
-      <c r="P7" s="44"/>
-      <c r="Q7" s="44"/>
-      <c r="R7" s="44" t="s">
-        <v>95</v>
-      </c>
-      <c r="S7" s="44"/>
-      <c r="T7" s="44"/>
-      <c r="U7" s="44"/>
-      <c r="V7" s="44"/>
-      <c r="W7" s="44" t="s">
-        <v>102</v>
-      </c>
-      <c r="X7" s="44"/>
+      <c r="M7" s="43"/>
+      <c r="N7" s="43"/>
+      <c r="O7" s="43"/>
+      <c r="P7" s="43"/>
+      <c r="Q7" s="43"/>
+      <c r="R7" s="43" t="s">
+        <v>93</v>
+      </c>
+      <c r="S7" s="43"/>
+      <c r="T7" s="43"/>
+      <c r="U7" s="43"/>
+      <c r="V7" s="43"/>
+      <c r="W7" s="43" t="s">
+        <v>100</v>
+      </c>
+      <c r="X7" s="43"/>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="20" t="s">
@@ -9402,10 +9401,10 @@
         <v>80</v>
       </c>
       <c r="J8" s="21" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="K8" s="21" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="L8" s="22" t="s">
         <v>54</v>
@@ -9420,31 +9419,31 @@
         <v>74</v>
       </c>
       <c r="P8" s="22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="Q8" s="23" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="R8" s="25" t="s">
+        <v>90</v>
+      </c>
+      <c r="S8" s="25" t="s">
+        <v>91</v>
+      </c>
+      <c r="T8" s="25" t="s">
         <v>92</v>
       </c>
-      <c r="S8" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="T8" s="25" t="s">
-        <v>94</v>
-      </c>
       <c r="U8" s="25" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="V8" s="25" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="W8" s="29" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="X8" s="30" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.2">
@@ -9452,7 +9451,7 @@
         <v>1</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="C9" s="3">
         <v>124</v>
@@ -9471,10 +9470,16 @@
       <c r="I9" s="3"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3" t="s">
-        <v>90</v>
-      </c>
-      <c r="L9" s="3"/>
-      <c r="M9" s="3"/>
+        <v>88</v>
+      </c>
+      <c r="L9" s="3">
+        <f>0.06*C9</f>
+        <v>7.4399999999999995</v>
+      </c>
+      <c r="M9" s="3">
+        <f>0.35*E9</f>
+        <v>420</v>
+      </c>
       <c r="N9" s="3"/>
       <c r="O9" s="3"/>
       <c r="P9" s="3"/>
@@ -10237,263 +10242,263 @@
         <v>-15</v>
       </c>
       <c r="D2" s="27" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="45" t="s">
+      <c r="A4" s="47" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="45"/>
-      <c r="D4" s="45" t="s">
+      <c r="B4" s="47"/>
+      <c r="D4" s="47" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="45"/>
-      <c r="G4" s="45" t="s">
+      <c r="E4" s="47"/>
+      <c r="G4" s="47" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="45"/>
-      <c r="J4" s="45" t="s">
+      <c r="H4" s="47"/>
+      <c r="J4" s="47" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="45"/>
-      <c r="M4" s="45" t="s">
+      <c r="K4" s="47"/>
+      <c r="M4" s="47" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="45"/>
-      <c r="P4" s="45" t="s">
+      <c r="N4" s="47"/>
+      <c r="P4" s="47" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="45"/>
+      <c r="Q4" s="47"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="45" t="s">
+      <c r="S4" s="47" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="45"/>
+      <c r="T4" s="47"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="45" t="s">
+      <c r="V4" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="45"/>
+      <c r="W4" s="47"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="45" t="s">
+      <c r="Y4" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="45"/>
+      <c r="Z4" s="47"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="45" t="s">
+      <c r="AB4" s="47" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="45"/>
-      <c r="AE4" s="45" t="s">
+      <c r="AC4" s="47"/>
+      <c r="AE4" s="47" t="s">
+        <v>114</v>
+      </c>
+      <c r="AF4" s="47"/>
+      <c r="AG4" s="1"/>
+      <c r="AH4" s="47" t="s">
+        <v>115</v>
+      </c>
+      <c r="AI4" s="47"/>
+      <c r="AJ4" s="1"/>
+      <c r="AK4" s="47" t="s">
         <v>116</v>
       </c>
-      <c r="AF4" s="45"/>
-      <c r="AG4" s="1"/>
-      <c r="AH4" s="45" t="s">
+      <c r="AL4" s="47"/>
+      <c r="AM4" s="1"/>
+      <c r="AN4" s="47" t="s">
         <v>117</v>
       </c>
-      <c r="AI4" s="45"/>
-      <c r="AJ4" s="1"/>
-      <c r="AK4" s="45" t="s">
+      <c r="AO4" s="47"/>
+      <c r="AP4" s="1"/>
+      <c r="AQ4" s="47" t="s">
         <v>118</v>
       </c>
-      <c r="AL4" s="45"/>
-      <c r="AM4" s="1"/>
-      <c r="AN4" s="45" t="s">
-        <v>119</v>
-      </c>
-      <c r="AO4" s="45"/>
-      <c r="AP4" s="1"/>
-      <c r="AQ4" s="45" t="s">
-        <v>120</v>
-      </c>
-      <c r="AR4" s="45"/>
+      <c r="AR4" s="47"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="B5" s="42">
         <v>1</v>
       </c>
       <c r="D5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E5" s="42">
         <v>2</v>
       </c>
       <c r="G5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="H5" s="42">
         <v>3</v>
       </c>
       <c r="J5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K5" s="42">
         <v>4</v>
       </c>
       <c r="M5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="N5" s="42">
         <v>5</v>
       </c>
       <c r="P5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="Q5" s="42">
         <v>6</v>
       </c>
       <c r="R5" s="1"/>
       <c r="S5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="T5" s="42">
         <v>7</v>
       </c>
       <c r="U5" s="1"/>
       <c r="V5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="W5" s="42">
         <v>8</v>
       </c>
       <c r="X5" s="1"/>
       <c r="Y5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="Z5" s="42">
         <v>9</v>
       </c>
       <c r="AA5" s="1"/>
       <c r="AB5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AC5" s="42">
         <v>10</v>
       </c>
       <c r="AE5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AF5" s="42">
         <v>11</v>
       </c>
       <c r="AG5" s="1"/>
       <c r="AH5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AI5" s="42">
         <v>12</v>
       </c>
       <c r="AJ5" s="1"/>
       <c r="AK5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AL5" s="42">
         <v>13</v>
       </c>
       <c r="AM5" s="1"/>
       <c r="AN5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AO5" s="42">
         <v>14</v>
       </c>
       <c r="AP5" s="1"/>
       <c r="AQ5" s="41" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="AR5" s="42">
         <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="46" t="str">
+      <c r="A6" s="45" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v>soil</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="D6" s="46" t="str">
+      <c r="B6" s="46"/>
+      <c r="D6" s="45" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="47"/>
-      <c r="G6" s="46" t="str">
+      <c r="E6" s="46"/>
+      <c r="G6" s="45" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="47"/>
-      <c r="J6" s="46" t="str">
+      <c r="H6" s="46"/>
+      <c r="J6" s="45" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="47"/>
-      <c r="M6" s="46" t="str">
+      <c r="K6" s="46"/>
+      <c r="M6" s="45" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="47"/>
-      <c r="P6" s="46" t="str">
+      <c r="N6" s="46"/>
+      <c r="P6" s="45" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="47"/>
+      <c r="Q6" s="46"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="46" t="str">
+      <c r="S6" s="45" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="47"/>
+      <c r="T6" s="46"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="46" t="str">
+      <c r="V6" s="45" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="47"/>
+      <c r="W6" s="46"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="46" t="str">
+      <c r="Y6" s="45" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="47"/>
+      <c r="Z6" s="46"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="46" t="str">
+      <c r="AB6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="47"/>
-      <c r="AE6" s="46" t="str">
+      <c r="AC6" s="46"/>
+      <c r="AE6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="47"/>
+      <c r="AF6" s="46"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="46" t="str">
+      <c r="AH6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="47"/>
+      <c r="AI6" s="46"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="46" t="str">
+      <c r="AK6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="47"/>
+      <c r="AL6" s="46"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="46" t="str">
+      <c r="AN6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="47"/>
+      <c r="AO6" s="46"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="46" t="str">
+      <c r="AQ6" s="45" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="47"/>
+      <c r="AR6" s="46"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -11413,36 +11418,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -11459,15 +11464,15 @@
   <sheetData>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A2" s="48" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B2" s="48"/>
       <c r="D2" s="49" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="E2" s="49"/>
       <c r="G2" s="24" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
@@ -12013,32 +12018,32 @@
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B2" s="50" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C2" s="50"/>
       <c r="D2" s="50"/>
       <c r="F2" s="50" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="G2" s="50"/>
       <c r="H2" s="50"/>
       <c r="J2" s="50" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K2" s="50"/>
       <c r="L2" s="50"/>
       <c r="N2" s="50" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="O2" s="50"/>
       <c r="P2" s="50"/>
       <c r="R2" s="50" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="S2" s="50"/>
       <c r="T2" s="50"/>
       <c r="V2" s="50" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="W2" s="50"/>
       <c r="X2" s="50"/>
@@ -12513,32 +12518,32 @@
   <sheetData>
     <row r="2" spans="2:24" x14ac:dyDescent="0.2">
       <c r="B2" s="51" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C2" s="51"/>
       <c r="D2" s="51"/>
       <c r="F2" s="51" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="G2" s="51"/>
       <c r="H2" s="51"/>
       <c r="J2" s="51" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="K2" s="51"/>
       <c r="L2" s="51"/>
       <c r="N2" s="51" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="O2" s="51"/>
       <c r="P2" s="51"/>
       <c r="R2" s="51" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="S2" s="51"/>
       <c r="T2" s="51"/>
       <c r="V2" s="51" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="W2" s="51"/>
       <c r="X2" s="51"/>

</xml_diff>